<commit_message>
tracker: store job descriptions as plain text, not markdown
update-application-tracker.py now strips markdown (headings, bold,
links, bullets) from jd.md before writing the Excel cell; existing
21 rows converted in place.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/application-tracker.xlsx
+++ b/application-tracker.xlsx
@@ -560,13 +560,13 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t># Machine Learning Engineer, Operations Technology
-**Location:** Toronto, Ontario, Canada
-**Company:** HelloFresh (HelloFresh Canada)
-**Pay Range (Toronto, ON):** $135,000 - $155,000 CAD
-**Work model:** Flexible Hybrid — minimum 2 days in office per week (most teams 2-3 days) · #LI-HYBRID
+          <t>Machine Learning Engineer, Operations Technology
+Location: Toronto, Ontario, Canada
+Company: HelloFresh (HelloFresh Canada)
+Pay Range (Toronto, ON): $135,000 - $155,000 CAD
+Work model: Flexible Hybrid — minimum 2 days in office per week (most teams 2-3 days) · #LI-HYBRID
 We are hiring a Machine Learning Engineer in our ML Solutions squad to help build innovative generative AI products that provide AI-powered assistants to HelloFresh's culinary Chefs helping them editorialize content, validate recipe data, detect issues, suggest corrections, and ideate. As a Machine Learning Engineer, you will primarily contribute to our agentic generative AI system that automates recipe content production, while also supporting the MLOps platform that enables data scientists across the company to develop, deploy, and monitor ML models at scale.
-## Lettuce share what this role will be responsible for
+Lettuce share what this role will be responsible for
 - Develop and maintain an agentic GenAI system that integrates with HelloFresh's culinary content pipeline (API development, LLM orchestration, image generation).
 - Design and implement production-grade AI Agent evaluations to measure quality, reliability, and performance of generative outputs.
 - Design and build scalable, production-grade ML systems capable of handling large datasets, complex model pipelines, and real-time API integrations.
@@ -575,14 +575,14 @@
 - Improve operational excellence through automation, monitoring, drift detection, and data quality practices.
 - Stay up-to-date on advancements in generative AI, agentic workflows, and MLOps tooling, and propose improvements to the team's development lifecycle.
 - All other duties, as assigned
-## Sound a-peeling? Here's what we're looking for
+Sound a-peeling? Here's what we're looking for
 - Strong software development skills in Python and SQL, including DevOps practices, test-driven development (TDD), spec-driven development, and fluency working with AI coding agents.
 - Hands-on experience building and maintaining production ML systems, including model serving, monitoring, and CI/CD pipelines.
 - Familiarity or interest in generative AI (LLMs, image generation, prompt engineering, agentic architectures).
 - Experience with modern MLOps tooling such as MLFlow, feature engineering, Kubernetes, and workflow orchestration (e.g., Prefect). Experience with PySpark and Databricks is a plus.
 - A passion for building developer tools and platforms that improve productivity and enable other teams to scale ML adoption.
 - Ability to communicate complex technical findings to both technical and non-technical stakeholders.
-## Let's cut to the cheese, this is why you'll love it here
+Let's cut to the cheese, this is why you'll love it here
 - Box Discount - Amazing discounts on 1 box per week! 75% discount on weekly HelloFresh and Chefs Plate meal kits AND 50% off weekly Factor meal box.
 - Health &amp; Wellness - Health &amp; Dental benefits from day 1, a Health Spending Account, unlimited access to the Headspace app to meet your self-care needs, and 25% discount on GoodLife fitness memberships!
 - Vacation &amp; PTO - Time off is also an important part of self-care! We offer generous vacation and PTO to help you create a good work-life balance.
@@ -591,13 +591,13 @@
 - Work Hard &amp; Have Fun - From team socials to engaging company days, you'll have plenty of opportunity to experience the fun!
 - Diversity &amp; Inclusion Initiatives - With impactful ERG's like FreshPride, Women Empowered and LIMES, we are committed to our diversity, equity &amp; inclusion efforts.
 - Food Puns - this one is kind of a big dill if you haven't already noticed. We even have some punny meeting room names!
-## Flexible Hybrid Approach
+Flexible Hybrid Approach
 At HelloFresh, we know that flexible work arrangements are essential in enabling you to do your best work, while balancing your personal and life needs. Offering remote work flexibility, along with the opportunity to interact and collaborate in the office are all a part of creating a great employee experience.
 To meet these needs, we are pleased to provide Flexible Hybrid work. Flexible Hybrid is a people-first approach that is based on choice, trust, personalization, and empowers teams to choose when and how often they work from the office and work from home, in addition to team days and company days. This means a minimum of 2 days in office per week, with most teams in office between 2-3 days a week.
 #LI-HYBRID
 HelloFresh Canada uses AI-integrated technology to help us process and evaluate applications more efficiently. This includes tools that screen and assess candidate qualifications based on the requirements for this role. While these tools assist our workflow, all final selection decisions are made by our hiring team.
 This is a posting for an existing vacancy. We are actively seeking to fill this position.
-**Toronto, ON Pay Range:** $135,000 - $155,000 CAD</t>
+Toronto, ON Pay Range: $135,000 - $155,000 CAD</t>
         </is>
       </c>
     </row>
@@ -622,36 +622,36 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t># AI Engineer (Speech and Audio Systems) — FGF Brands
-**Primary Job Location:** CA-ON-Greater Toronto Area
-**Posted Date:** 3 hours ago (7/7/2026 5:37 AM)
-**Job Family:** IT
-**Job Type:** Full Time
-**Hours of Work:** Monday to Friday (normal operating hours)
-## Job Description
+          <t>AI Engineer (Speech and Audio Systems) — FGF Brands
+Primary Job Location: CA-ON-Greater Toronto Area
+Posted Date: 3 hours ago (7/7/2026 5:37 AM)
+Job Family: IT
+Job Type: Full Time
+Hours of Work: Monday to Friday (normal operating hours)
+Job Description
 AI Engineer (Speech and Audio Systems)
 We're a naan traditional company…
-### Job Summary:
+Job Summary:
 We are seeking a motivated, detail-oriented AI Engineer to join our growing Audio Intelligence team. In this role, you will help build, refine, and deploy machine learning models that understand human speech and sound. You will bridge the gap between creative audio engineering and deep learning by processing raw audio datasets, evaluating model performance, and helping us build the next generation of voice-activated technology.
-### What FGF Offers:
+What FGF Offers:
 - FGF believes in Home Grown Talent, accelerated career growth with leadership training. Unleashing Your Potential
 - Competitive Compensation, Health Benefits, &amp; a generous flexible medical / Health spending account
 - RRSP matching program
 - Tuition reimbursement
 - Discount program that covers almost everything under the sun - Restaurants, gyms, shopping etc.
-### Responsibilities:
-- **Data Curation &amp; Preprocessing:** Clean, segment, and format audio datasets for model training (handling noise reduction, volume normalization, and formatting).
-- **Audio Analysis &amp; Visual Inspection:** Use advanced spectral editing software to inspect, clean, and isolate specific sound events or speech anomalies in our training data.
-- **Model Training Support:** Assist in fine-tuning state-of-the-art automatic speech recognition (ASR) and audio classification models.
-- **Evaluation &amp; Benchmarking:** Run validation tests on trained models, track performance metrics (like Word Error Rate), and document failures to help guide future improvements.
-- **Collaboration:** Work closely with senior AI scientists and data engineering teams to maintain high-quality data pipelines.
-### Qualifications:
+Responsibilities:
+- Data Curation &amp; Preprocessing: Clean, segment, and format audio datasets for model training (handling noise reduction, volume normalization, and formatting).
+- Audio Analysis &amp; Visual Inspection: Use advanced spectral editing software to inspect, clean, and isolate specific sound events or speech anomalies in our training data.
+- Model Training Support: Assist in fine-tuning state-of-the-art automatic speech recognition (ASR) and audio classification models.
+- Evaluation &amp; Benchmarking: Run validation tests on trained models, track performance metrics (like Word Error Rate), and document failures to help guide future improvements.
+- Collaboration: Work closely with senior AI scientists and data engineering teams to maintain high-quality data pipelines.
+Qualifications:
 - Bachelor's degree in Computer Science, Data Science, Electrical/Audio Engineering, or a related technical field
 - Understanding of basic digital audio concepts like sampling rates, bit depth, channels, etc.
 - Familiarity with sound processing software such as SpectraLayers, Audacity, and python libraries such as scipy.signal, pydub, etc.
 - Strong foundational programming skills, familiarity with version control Git and software engineering best practices
 - Prior experience working in a fast-paced, high-growth environment (big tech or startup experience preferred).
-### What is the recipe for a great career at FGF?
+What is the recipe for a great career at FGF?
 Working at FGF Brands, there is never a dull moment! As a successful company that is continually growing there is always challenging yet rewarding work to be a part of. We have an entrepreneurial spirit which encourages all our team members to use their own creativity and out of the box thinking to come up with solutions and new ideas.
 In compliance with Ontario's Bill 190, we confirm that this posting represents a current, existing vacancy within our organization.
 Disclaimer: The above describes the general responsibilities, required knowledge and skills. Please keep in mind that other duties may be added or this description may be amended at any time.</t>
@@ -679,8 +679,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-AI Engineer
+          <t>AI Engineer
 About Armilla AI
 Armilla AI is a cutting-edge startup based in Toronto, Ontario, Canada, operating at the intersection of artificial intelligence and insurance. We're not just talking about AI risk; we're actively building the solutions to manage, underwrite, and insure it. Our dynamic team is passionate about pioneering the future of AI risk management through the development of sophisticated AI-powered tools and programmatic evaluation platforms.
 The Role: Building &amp; Evaluating AI Solutions
@@ -742,8 +741,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-JOB ID -SAPXJP00084142
+          <t>JOB ID -SAPXJP00084142
 Request Title
 Developer T2 (CAN)
 Description
@@ -798,8 +796,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-Software Developer
+          <t>Software Developer
 Apply
 locations
 UBC Vancouver Campus - Vancouver, BC, Canada
@@ -906,7 +903,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t># Full Stack Developer Intern (Fall 2026) — GeoComply
+          <t>Full Stack Developer Intern (Fall 2026) — GeoComply
 Vancouver, BC
 Customer – Revenue /
 Intern /
@@ -916,69 +913,69 @@
 Application deadline: July 23, 2026
 Salary range: $54,000 and ~$62,000 (annualized, prorated to your ~4-month placement).
 We're GeoComply, an identity verification, anti-fraud and compliance company that uses advanced location detection and device intelligence to verify user identity and catch fraud online before loss happens.
-## The problem you'd be working on:
+The problem you'd be working on:
 When a GeoComply client wants to understand a fraud decision our systems made, or change how one of their rules resolves, it's a black box on the client side. They ask us, we make the changes, and the client never really sees exactly how their data moved through our pipeline or why a given outcome fired.
 We want to fix that by building a customer-facing system inside our product that ingests transaction data, shows our customers where each signal flows through our pipeline, and lets them tune rule outcomes themselves.
 Over four months, your job will be to help turn a prototype into something we can put in front of real clients and grow toward a production feature that will make a lasting impact on how hundreds of our customers use us as a tool in their verification, anti-fraud, and compliance arsonals.
-## Key Responsibilities
-* Build features on a real product: the UI that makes our decisioning visible, and the ingestion and API work behind it.
-* Get operator event data flowing in (Segment events, analytics SDKs, webhooks) and reason about the full loop: ingest, enrich, decide, act.
-* Dig into how rules and signals actually work today and figure out how to expose that to a customer safely, and in a way that they can digest, not just with information overload.
-* Sit close to real client conversations (we're already lining up demos), take the feedback, and fold it back into what you build.
-* Use AI the way this team already does: to move faster, clear your own blockers, and build things a senior developer couldn't ship a few years ago.
-## Role Requirements
-* Current students preferred; your specific degree doesn't matter, as long as you have the full-stack skills, interests, and aptitude we're looking for.
-* You're familiar with APIs, event data, and integrations, and you can pick up an unfamiliar codebase with minimal despair.
-* You're strong in React and TypeScript, or strong enough elsewhere that you can get there fast.
-* You've written a real backend in something (Python is a plus).
-* You can look at something messy and undocumented, ask a lot of sharp questions, and build a clear picture.
-* You handle data carefully. When it's a real transaction and personal data, your attention to detail will matter more than speed.
-* You can talk to non-engineers, including customers and even our Executive Leadership Team, and explain why your work matters in their language.
-* Embrace Stretch Opportunities (The Fun Part!): As a GeoComply intern, expect to be pushed. You'll be given special, high-value projects outside the immediate scope of your role; a chance to explore new skills, test your limits, and adapt to new challenges across the business.
-## Why the right person will love this role:
-* You're working on a real product with real customers and revenue riding on it. If successful, your code will be seen (and hopefully loved!) by our customers.
-* The problem is meaty and cross-disciplinary: data, fraud, ML, and customer trust in one build.
-* Exposure to Fraud, Risk, and Trust and Safety use cases: account takeover, bonus abuse, multi-account rings, proxy and device spoofing, and the million other patterns we help our clients fight every day.
-* Visibility to customers and end users by default.
-## You'll get your hands on the guts of how GeoComply catches fraud:
-* Prototypes and the wider Risk Platform it's growing into.
-* Event ingestion: Segment, analytics SDKs, webhooks, and the pipelines that carry operator transaction data.
-* Databricks and the data platform where all of this lands.
-* The rule engine world: how fraud rules, signals, and configs actually resolve, including the shadow-mode and adaptive-config machinery most people never see.
-* GeoComply's product suite up close: RiskGuard's signals, IDComply's identity checks, and our decisioning layers.
-* AI tooling as a daily building partner, which is already how this team works.
-## You'll hate this role if you can't handle:
-* A lack of clean specs, shifting scope. Someone who needs a defined backlog may feel unmoored, and someone who wants tidy docs and one person handing them end to end tasks will stall.
-* Customer, internal teams, and live demo/feedback exposure. Someone who wants to code alone in a corner will dread the required stakeholder load.
-* High-consequence domain: fraud, compliance, PII, production-adjacent data. Someone careless, or who wants a low-stakes sandbox is a bad fit.
-## How mentorship and support work
+Key Responsibilities
+- Build features on a real product: the UI that makes our decisioning visible, and the ingestion and API work behind it.
+- Get operator event data flowing in (Segment events, analytics SDKs, webhooks) and reason about the full loop: ingest, enrich, decide, act.
+- Dig into how rules and signals actually work today and figure out how to expose that to a customer safely, and in a way that they can digest, not just with information overload.
+- Sit close to real client conversations (we're already lining up demos), take the feedback, and fold it back into what you build.
+- Use AI the way this team already does: to move faster, clear your own blockers, and build things a senior developer couldn't ship a few years ago.
+Role Requirements
+- Current students preferred; your specific degree doesn't matter, as long as you have the full-stack skills, interests, and aptitude we're looking for.
+- You're familiar with APIs, event data, and integrations, and you can pick up an unfamiliar codebase with minimal despair.
+- You're strong in React and TypeScript, or strong enough elsewhere that you can get there fast.
+- You've written a real backend in something (Python is a plus).
+- You can look at something messy and undocumented, ask a lot of sharp questions, and build a clear picture.
+- You handle data carefully. When it's a real transaction and personal data, your attention to detail will matter more than speed.
+- You can talk to non-engineers, including customers and even our Executive Leadership Team, and explain why your work matters in their language.
+- Embrace Stretch Opportunities (The Fun Part!): As a GeoComply intern, expect to be pushed. You'll be given special, high-value projects outside the immediate scope of your role; a chance to explore new skills, test your limits, and adapt to new challenges across the business.
+Why the right person will love this role:
+- You're working on a real product with real customers and revenue riding on it. If successful, your code will be seen (and hopefully loved!) by our customers.
+- The problem is meaty and cross-disciplinary: data, fraud, ML, and customer trust in one build.
+- Exposure to Fraud, Risk, and Trust and Safety use cases: account takeover, bonus abuse, multi-account rings, proxy and device spoofing, and the million other patterns we help our clients fight every day.
+- Visibility to customers and end users by default.
+You'll get your hands on the guts of how GeoComply catches fraud:
+- Prototypes and the wider Risk Platform it's growing into.
+- Event ingestion: Segment, analytics SDKs, webhooks, and the pipelines that carry operator transaction data.
+- Databricks and the data platform where all of this lands.
+- The rule engine world: how fraud rules, signals, and configs actually resolve, including the shadow-mode and adaptive-config machinery most people never see.
+- GeoComply's product suite up close: RiskGuard's signals, IDComply's identity checks, and our decisioning layers.
+- AI tooling as a daily building partner, which is already how this team works.
+You'll hate this role if you can't handle:
+- A lack of clean specs, shifting scope. Someone who needs a defined backlog may feel unmoored, and someone who wants tidy docs and one person handing them end to end tasks will stall.
+- Customer, internal teams, and live demo/feedback exposure. Someone who wants to code alone in a corner will dread the required stakeholder load.
+- High-consequence domain: fraud, compliance, PII, production-adjacent data. Someone careless, or who wants a low-stakes sandbox is a bad fit.
+How mentorship and support work
 Your manager is our Director of Engineering who sits in the Vancouver office, she'll also be your technical mentor day to day. You'll also work alongside the senior engineers who built the Risk Platform and the product and leadership people deciding where it goes next, so the feedback you get comes from the people making the real calls.
 On top of your team, you're part of the Early Talent cohort: structured check-ins, a group of other interns chewing on hard problems next to you, and skip-level time with senior leadership built into the program.
 If your manager is away for a week, the scaffolding around you will be there to bridge the gap.
-## What You'll Gain
-* Ownership of a product with customers and revenue attached, and the rare intern experience of taking something from prototype toward production.
-* Hands-on experience and mentorship in a stack most new grads never touch: event pipelines, a live rule engine, data platforms, and the anti-fraud domain behind them.
-* Proof you can build. If this lands, your work goes in front of real clients, and you can point at it long after the term ends.
-* A front-row view of how fraud, data, and product decisions get made at a company protecting some of the biggest names in gaming and finance.
-* Support and feedback from senior engineers and leaders who treat interns as builders, disruptors, and innovators, not helpers or coffee-runners.
-## Bonus Points if (nice to have, not needed)
-* React Flow, Monaco, or other rich interactive-UI libraries
-* FastAPI or another Python web framework
-* WebSockets / real-time streaming, or event pipelines (Segment, webhooks)
-* Docker, GCP, or Postgres
-* Any exposure to fraud, risk, or data visualization.
+What You'll Gain
+- Ownership of a product with customers and revenue attached, and the rare intern experience of taking something from prototype toward production.
+- Hands-on experience and mentorship in a stack most new grads never touch: event pipelines, a live rule engine, data platforms, and the anti-fraud domain behind them.
+- Proof you can build. If this lands, your work goes in front of real clients, and you can point at it long after the term ends.
+- A front-row view of how fraud, data, and product decisions get made at a company protecting some of the biggest names in gaming and finance.
+- Support and feedback from senior engineers and leaders who treat interns as builders, disruptors, and innovators, not helpers or coffee-runners.
+Bonus Points if (nice to have, not needed)
+- React Flow, Monaco, or other rich interactive-UI libraries
+- FastAPI or another Python web framework
+- WebSockets / real-time streaming, or event pipelines (Segment, webhooks)
+- Docker, GCP, or Postgres
+- Any exposure to fraud, risk, or data visualization.
 $54,000 - $62,000 a year
-## Why is our salary range so large?
+Why is our salary range so large?
 This role pays between $54,000 and ~$62,000 (annualized, prorated to your ~4-month placement). That's a wide band, and we'd rather explain it than pretend it isn't.
 The range covers every technical intern we hire across three variables: whether this is your first product internship or your third+, whether you're at the beginning of your Bachelor's or at the end of your Master's, and actually extends beyond that for more senior / PhD or MBA level candidates who come into the Early Talent Program.
 TL;DR: A first-internship bachelor's student and a Master's student with two years of work experience are both encouraged to apply: they just won't be paid the same, and they shouldn't be.
-## About GeoComply's Early Talent Program
+About GeoComply's Early Talent Program
 Most companies see interns as cheap labour, a temporary workforce, or someone to hand the tasks nobody else wants. We think that's a huge missed opportunity.
 GeoComply treats our Early Talent Program as a chance to hand-select and shape our future leaders: to give them the roots of the skills we want our team leads to have in five years, and our executives in fifteen. We develop our future pipeline of people as thoughtfully as we develop our products.
 The stats back that up:
-* GeoComply supports an average of 60 intern positions a year, globally.
-* 8 to 10% of our current workforce were hired on as interns.
-* Every intern gets hundreds of hours of job-specific training and professional development from their managers, mentors, and the Early Talent Program.
+- GeoComply supports an average of 60 intern positions a year, globally.
+- 8 to 10% of our current workforce were hired on as interns.
+- Every intern gets hundreds of hours of job-specific training and professional development from their managers, mentors, and the Early Talent Program.
 Learn more about the program and our benefits: https://www.geocomply.com/careers/internship/
 Not sure you qualify for this role? Apply anyway. At GeoComply, Passion, Hunger, and Drive (aka PhD) count for more than relevant experience or a specific skill set.
 Our workplace is built on mutual respect and inclusion. We know that diversity of experience and thought drives connection, innovation, and our success, and we welcome applicants of all backgrounds, experiences, beliefs, and identities.
@@ -1007,38 +1004,36 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-Business Intelligence &amp; Analytics Specialist
+          <t>Business Intelligence &amp; Analytics Specialist
 Job Category: Information Technology
 Requisition Number: BIDEV002488
 Posting Details
-*
-* Posted: July 9, 2026
-* Full-Time
-* Hybrid
-* Locations
+- - Posted: July 9, 2026
+- Full-Time
+- Hybrid
+- Locations
 Showing 1 location
 Nature's Path Foods Richmond, BC V6X1W3, CAN
 Job Details
 Description
 Key Responsibilities
-* Business Engagement &amp; Requirements: Partner with Sales, Finance, and Supply Chain to understand processes and KPIs, lead requirements sessions, and translate business needs into clear analytical solutions.
-* Development &amp; Delivery: Build and maintain Power BI solutions, including intuitive reports and dashboards, wireframes, semantic models, and advanced DAX within Microsoft Fabric.
-* Problem Solving &amp; Analysis: Break down complex requests, investigate data discrepancies, ensure reporting accuracy, and drive automation and process improvements.
+- Business Engagement &amp; Requirements: Partner with Sales, Finance, and Supply Chain to understand processes and KPIs, lead requirements sessions, and translate business needs into clear analytical solutions.
+- Development &amp; Delivery: Build and maintain Power BI solutions, including intuitive reports and dashboards, wireframes, semantic models, and advanced DAX within Microsoft Fabric.
+- Problem Solving &amp; Analysis: Break down complex requests, investigate data discrepancies, ensure reporting accuracy, and drive automation and process improvements.
 Required Qualifications
-* Bachelor's degree (or equivalent) in Computer Science, Analytics, or a related field.
-* Minimum 4 years of experience in a BI or analytics role.
-* Strong hands-on experience with Power BI and Microsoft Fabric.
-* Proficiency in SQL, data modeling, and DAX.
-* Experience with row-level security, column-level filtering, role-based access controls, and data masking/anonymization.
+- Bachelor's degree (or equivalent) in Computer Science, Analytics, or a related field.
+- Minimum 4 years of experience in a BI or analytics role.
+- Strong hands-on experience with Power BI and Microsoft Fabric.
+- Proficiency in SQL, data modeling, and DAX.
+- Experience with row-level security, column-level filtering, role-based access controls, and data masking/anonymization.
 Preferred Qualifications
-* Experience in the Consumer Packaged Goods (CPG) industry.
-* Knowledge of (or willingness to learn) data architecture, ETL, and data engineering using Python/PySpark.
-* Microsoft Fabric Analytics Engineer or Power BI certification.
-* Familiarity with ERP data.
+- Experience in the Consumer Packaged Goods (CPG) industry.
+- Knowledge of (or willingness to learn) data architecture, ETL, and data engineering using Python/PySpark.
+- Microsoft Fabric Analytics Engineer or Power BI certification.
+- Familiarity with ERP data.
 Notes
-* Salary range: $85,000–$100,000, plus a 10% bonus.
-* This role is based in the Richmond office 4 days per week.</t>
+- Salary range: $85,000–$100,000, plus a 10% bonus.
+- This role is based in the Richmond office 4 days per week.</t>
         </is>
       </c>
     </row>
@@ -1063,13 +1058,13 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t># AI/ML Platform Developer (Contract) — via Apex Systems
-**Client:** SAP
-**Location:** Vancouver, BC, Canada (Hybrid — 3x per week onsite)
-**Duration:** 12-month Contract
-**Recruiter:** Jessica Nagra, Technical Recruiter, Apex Systems
-**Setup:** Incorporated (corp-to-corp), $37–40/hr, no benefits or PTO (T4 option to be confirmed on call)
-## What You Will Build
+          <t>AI/ML Platform Developer (Contract) — via Apex Systems
+Client: SAP
+Location: Vancouver, BC, Canada (Hybrid — 3x per week onsite)
+Duration: 12-month Contract
+Recruiter: Jessica Nagra, Technical Recruiter, Apex Systems
+Setup: Incorporated (corp-to-corp), $37–40/hr, no benefits or PTO (T4 option to be confirmed on call)
+What You Will Build
 Our client, a Fortune 500 global enterprise software and ERP platform provider, is looking for an AI/ML Platform Developer to join their Business Data Cloud Foundation Infrastructure organization. In this role, you will design, implement, and operate the cloud-native infrastructure that powers our client's next-generation Business Data Cloud solutions.
 You will:
 - Collaborate with engineering and operations to design and maintain build systems, CI/CD pipelines, and deployment tooling.
@@ -1078,7 +1073,7 @@
 - Translate complex requirements from cross-functional stakeholders into technical designs and executable implementation plans.
 - Lead design reviews, produce clear technical documentation, provide peer feedback, and represent your work through demos, presentations, and retrospectives.
 - Contribute to the client's intelligent technology portfolio by enabling reliable, data-driven decision making at scale.
-## What You Bring
+What You Bring
 - 1–2 years of hands-on experience in SRE/DevOps, systems engineering, cloud operations, or automation in enterprise environments.
 - Proficiency in cloud platforms (AWS, GCP, Azure, or enterprise BTP-equivalent) and container technologies (Kubernetes, Cloud Foundry, Docker, cloud databases, and data/event pipelines).
 - Experience building and operating complex CI/CD pipelines (e.g., Jenkins, Argo CD, Flux CD, GitHub Actions) and automated delivery processes.
@@ -1086,17 +1081,17 @@
 - Ability to write maintainable, production-grade code in languages such as Python, Java, or similar.
 - Excellent communication skills with the ability to articulate technical concepts to both technical and non-technical audiences.
 - Bachelor's degree in computer science, Engineering, or equivalent work experience.
-## Preferred Qualifications
+Preferred Qualifications
 - Experience designing highly available, horizontally scalable distributed systems, including traffic management, autoscaling, and progressive delivery patterns.
 - Ability to architect modular, reusable distributed systems.
 - Experience implementing Generative AI services, ML Ops tooling, or AI-driven enterprise applications.
 - Curiosity, a continuous-learning mindset, and a passion for knowledge-sharing.
 - Master's degree or equivalent experience.
-## EEO Employer
+EEO Employer
 Apex Systems is an equal opportunity employer. We do not discriminate or allow discrimination on the basis of race, color, religion, creed, sex (including pregnancy, childbirth, breastfeeding, or related medical conditions), age, sexual orientation, gender identity, national origin, ancestry, citizenship, genetic information, registered domestic partner status, marital status, disability, status as a crime victim, protected veteran status, political affiliation, union membership, or any other characteristic protected by law. Apex will consider qualified applicants with criminal histories in a manner consistent with the requirements of applicable law. If you have visited our website in search of information on employment opportunities or to apply for a position, and you require an accommodation in using our website for a search or application, please contact our Employee Services Department at employeeservices@apexsystems.com or 844-463-6178.
-## Notes
+Notes
 - Official JD docx received from Apex 2026-07-15 ("AI ML Platform Developer JD.docx"); its content matches this reconstruction verbatim, plus the EEO statement above. The official posting contains NO rate/incorporation/T4 terms — those come only from Jessica Nagra's email ($40/hr INC, no benefits/PTO).
-- Same client (SAP) and near-identical role as the Vaco-sourced "Developer T2 (Platform Eng &amp; AI/ML)" (req SAPXJP00084142). User is pursuing via Apex and withdrawing from Vaco. Reuse the SAP materials on branch `2026-07-13-sap-platform-developer`.</t>
+- Same client (SAP) and near-identical role as the Vaco-sourced "Developer T2 (Platform Eng &amp; AI/ML)" (req SAPXJP00084142). User is pursuing via Apex and withdrawing from Vaco. Reuse the SAP materials on branch 2026-07-13-sap-platform-developer.</t>
         </is>
       </c>
     </row>
@@ -1121,44 +1116,43 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-Data Scientist, Analytics (Remote, Canada)
+          <t>Data Scientist, Analytics (Remote, Canada)
 Remote (Canada)
 Data Scientist, Analytics
 (Remote, Canada)
 Events in recent years have made us all too familiar with the havoc that natural disasters can wreak, and the increasing frequency and intensity with which they are occurring. Despite record levels of losses, conventional methods of risk modeling continue to paint at best an incomplete picture of these threats.
-[ZestyAI](http://zesty.ai/) uses novel data gathering and data science methods to produce higher quality information about the risks to property from catastrophes like storms and wildfires. While AI alone may not be able to thwart these disasters, it can help us become more prepared for them, and ultimately that will lead to better outcomes.
+ZestyAI uses novel data gathering and data science methods to produce higher quality information about the risks to property from catastrophes like storms and wildfires. While AI alone may not be able to thwart these disasters, it can help us become more prepared for them, and ultimately that will lead to better outcomes.
 As a Data Scientist, Analytics, you will work closely with product, engineering, and machine learning teams to apply data science to complex product and business problems. You will use diverse data sources to evaluate product performance, generate actionable insights, and support evidence-based decision-making across ZestyAI's products. You will also help establish the analytical processes, monitoring frameworks, and best practices needed to maintain product quality and scale the organization. You thrive in a collaborative, creative environment that moves fast and are comfortable implementing structures and processes to help the company scale.
 The Opportunity:
-* Translate product management, engineering, and business questions into structured analytical approaches, applying appropriate statistical, experimental, and data science methods to measure product performance and guide decision-making
-* Own data quality of ZestyAI data products
-* Spearhead product monitoring and quality assurance by designing and owning dashboards and KPIs
-* Develop automated ETL and data workflows
-* Iterate rapidly on everything; all of the above happens in a fast-paced business-driven environment that you must be comfortable with
-What You Bring to the [ZestyAI](http://zesty.ai/) Team:
-* BA / BS degree in Math, Physics, Engineering, Computer Science, or Economics
-   * MS or Ph.D. is certainly a bonus
-* 2–3 years of experience in analytics, data science, or related roles, including experience building data workflows, defining metrics, and developing dashboards or monitoring tools
-* Strong organizational and management skills with past experiences implementing best practices and processes
-* Strong analytical problem-solving skills and comfort working with ambiguous, cross-functional questions
-* Proficient in SQL
-* Proficient in programming language (Python or R)
-* Experience working with cloud platforms (Google Cloud Platform, AWS, etc)
-* Must be legally eligible to work in Canada
+- Translate product management, engineering, and business questions into structured analytical approaches, applying appropriate statistical, experimental, and data science methods to measure product performance and guide decision-making
+- Own data quality of ZestyAI data products
+- Spearhead product monitoring and quality assurance by designing and owning dashboards and KPIs
+- Develop automated ETL and data workflows
+- Iterate rapidly on everything; all of the above happens in a fast-paced business-driven environment that you must be comfortable with
+What You Bring to the ZestyAI Team:
+- BA / BS degree in Math, Physics, Engineering, Computer Science, or Economics
+   - MS or Ph.D. is certainly a bonus
+- 2–3 years of experience in analytics, data science, or related roles, including experience building data workflows, defining metrics, and developing dashboards or monitoring tools
+- Strong organizational and management skills with past experiences implementing best practices and processes
+- Strong analytical problem-solving skills and comfort working with ambiguous, cross-functional questions
+- Proficient in SQL
+- Proficient in programming language (Python or R)
+- Experience working with cloud platforms (Google Cloud Platform, AWS, etc)
+- Must be legally eligible to work in Canada
 Nice to Have:
-* 1 - 2 years of experience working with imagery and/or geospatial data
-* Working knowledge of modeling framework and performance metrics
-* Familiarity with, or an interest in, experimental design, causal inference, and applied statistical methods
-* DBT Experience
-* Prefect (or another workflow tool like Airflow) Experience
-* Data Visualization Experience
-Why [ZestyAI](http://zesty.ai/):
-* Be part of a well-funded growth-stage company
-* Market competitive comp and equity incentives to give you a stake in our future
-* Comprehensive health care plan
-* Flexible Time Off
-* An upbeat and collaborative work culture
-* Company-sponsored outings and offsites</t>
+- 1 - 2 years of experience working with imagery and/or geospatial data
+- Working knowledge of modeling framework and performance metrics
+- Familiarity with, or an interest in, experimental design, causal inference, and applied statistical methods
+- DBT Experience
+- Prefect (or another workflow tool like Airflow) Experience
+- Data Visualization Experience
+Why ZestyAI:
+- Be part of a well-funded growth-stage company
+- Market competitive comp and equity incentives to give you a stake in our future
+- Comprehensive health care plan
+- Flexible Time Off
+- An upbeat and collaborative work culture
+- Company-sponsored outings and offsites</t>
         </is>
       </c>
     </row>
@@ -1183,8 +1177,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-Software Development Engineer, Middle Mile P&amp;O
+          <t>Software Development Engineer, Middle Mile P&amp;O
 Job ID: 3185274 | Amazon Development Centre Canada ULC
 Description
 The Route Execution Optimization (REO) team in Middle Mile Planning and Optimization (MMPO) is seeking a Software Development Engineer II to build systems that automatically respond to transportation network disruptions—weather delays, facility closures, equipment failures, and driver constraints. You'll design intent-based automation that orchestrates optimal route corrections while maintaining safety, compliance, and efficiency. This role offers the opportunity to solve complex distributed systems challenges at massive scale, affecting hundreds of thousands of loads weekly, directly reducing operational costs and improving driver safety across Amazon's middle-mile transportation network.
@@ -1242,11 +1235,10 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-Data Analyst EA SPORTS™ FC (Game Development Analytics)
-* [Home](https://jobs.ea.com/en_US/careers/Home)
-* [Open Roles](https://jobs.ea.com/en_US/careers/SearchJobs?jr_id=6a5e4f97050c423c792ee66a)
-* Role Detail
+          <t>Data Analyst EA SPORTS™ FC (Game Development Analytics)
+- Home
+- Open Roles
+- Role Detail
 General Information
 Locations: Vancouver, British Columbia, Canada
 Role ID
@@ -1265,33 +1257,33 @@
 As a Data Analyst you will play a key role in analyzing our operational data to improve our Quality Verification strategies for the EA Sports titles (such as FC, NBA and NHL). You should be a sharp, curious, and analytic individual who has a passion for diving into data to solve business problems. Your insights will influence how we build and verify the quality of our games, and how to improve our business processes through data insights.
 The Data Analyst will be responsible for assembling data from multiple sources, conducting analyses, performing research, interacting with different internal customers, designing, documenting, and implementing analytical solutions, as well as compiling and presenting results, in graphical and written summaries, to a variety of audiences. You will be responsible for building metrics reporting systems and for tracking process improvements across the organization. You will excel in a fast paced environment, managing multiple responsibilities and deadlines in an internationally based team. The ideal candidate would be an effective communicator who combines solid technical skills with pride in excellence, who also demonstrates the potential to grow into a client-facing consulting role and/or an analytical consulting role (i.e. development of simulation models).
 What a Data Analyst does at EA:
-* Assembles data from multiple sources, conducts analyses, performs research, designs, documents and implements analytical solutions.
-* Presents analysis conclusions to the internal customer in a clear, understandable, and valuable way.
-* Communicates with team members and business stakeholders.
-* Presents high quality reports and findings in Power BI or as presentations.
-* Builds metrics reporting systems and tracks process improvements across the team.
-* Conducts analysis using statistical software, databases, spreadsheets, and reporting tools
-* Designs, evaluate and monitor key metrics, understanding root causes of changes in metrics
-* Develops and maintains scripts and queries to import, manipulate, clean, transform data from different sources
-* Builds and shares live dashboards and reports complete with user documentation
-* Builds and trains statistical models for hypothesis testing
-* Performs quality assurance on generated results to ensure accuracy and consistency
-* Presents conclusions in a clear and concise way
+- Assembles data from multiple sources, conducts analyses, performs research, designs, documents and implements analytical solutions.
+- Presents analysis conclusions to the internal customer in a clear, understandable, and valuable way.
+- Communicates with team members and business stakeholders.
+- Presents high quality reports and findings in Power BI or as presentations.
+- Builds metrics reporting systems and tracks process improvements across the team.
+- Conducts analysis using statistical software, databases, spreadsheets, and reporting tools
+- Designs, evaluate and monitor key metrics, understanding root causes of changes in metrics
+- Develops and maintains scripts and queries to import, manipulate, clean, transform data from different sources
+- Builds and shares live dashboards and reports complete with user documentation
+- Builds and trains statistical models for hypothesis testing
+- Performs quality assurance on generated results to ensure accuracy and consistency
+- Presents conclusions in a clear and concise way
 The next great Data Analyst needs:
-* Relevant experience in a past analytical role.
-* Expert data visualization techniques for charts and reports - good knowledge of Microsoft Power BI and/or Tableau.
-* Unstructured Data handling - Know best practices on how to stage unstructured data and properly model it to solve the problem at hand
-* Must have very good database and SQL knowledge, NoSQL and elastic search - a strong bonus.
-* Data Analysis - good knowledge of R language, MS Excel mastery, including VBA, PivotTables, and array functions - or other similar tools used for discovering data patterns and correlations through statistical methods.
-* Good math and analytical skills including statistics, simulation, and optimization.
+- Relevant experience in a past analytical role.
+- Expert data visualization techniques for charts and reports - good knowledge of Microsoft Power BI and/or Tableau.
+- Unstructured Data handling - Know best practices on how to stage unstructured data and properly model it to solve the problem at hand
+- Must have very good database and SQL knowledge, NoSQL and elastic search - a strong bonus.
+- Data Analysis - good knowledge of R language, MS Excel mastery, including VBA, PivotTables, and array functions - or other similar tools used for discovering data patterns and correlations through statistical methods.
+- Good math and analytical skills including statistics, simulation, and optimization.
 We Thought You Might Also Want to Know:
-* Where are we located? The EA Vancouver Office is located in suburban Burnaby, British Columbia
-* EA is an equal opportunity employer. All employment decisions are made without regard to race, color, national origin, ancestry, sex, gender, gender identity or expression, sexual orientation, age, genetic information, religion, disability, medical condition, pregnancy, marital status, family status, veteran status, or any other characteristic protected by law. EA also makes workplace accommodations for qualified individuals with disabilities as required by applicable law.
+- Where are we located? The EA Vancouver Office is located in suburban Burnaby, British Columbia
+- EA is an equal opportunity employer. All employment decisions are made without regard to race, color, national origin, ancestry, sex, gender, gender identity or expression, sexual orientation, age, genetic information, religion, disability, medical condition, pregnancy, marital status, family status, veteran status, or any other characteristic protected by law. EA also makes workplace accommodations for qualified individuals with disabilities as required by applicable law.
 Pay Transparency - North America
 COMPENSATION AND BENEFITS
 The ranges listed below are what EA in good faith expects to pay applicants for this role in these locations at the time of this posting. If you reside in a different location, a recruiter will advise on the applicable range and benefits. Pay offered will be determined based on a number of relevant business and candidate factors (e.g. education, qualifications, certifications, experience, skills, geographic location, or business needs).
 PAY RANGES
-* British Columbia (depending on location e.g. Vancouver vs. Victoria) *$77,700 - $107,900 CAD
+ British Columbia (depending on location e.g. Vancouver vs. Victoria) $77,700 - $107,900 CAD
 Pay is just one part of the overall compensation at EA.
 In Canada, we offer a package of benefits including vacation (3 weeks per year to start), 10 days per year of sick time, and extended health/dental/vision coverage and basic life insurance.
 About Electronic Arts
@@ -1322,7 +1314,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t># Job Description (raw, verbatim)
+          <t>Job Description (raw, verbatim)
 Software Developer III
 Req #23574
 Canada
@@ -1334,25 +1326,25 @@
 About the Opportunity
 We are building the next generation of how customers are implemented in Dayforce. This team is transforming a massively complex process into one that can be led by customers, partners, and Dayforce employees with the support of both generative and non-generative AI. If you are energized by solving meaningful product and engineering problems, improving how work gets done, and helping shape AI-powered experiences that scale, this is an opportunity to make a real impact. This is an intermediate-level role where you'll own well-scoped features and components within a service, delivering solid execution on moderately complex problems while partnering with your team when requirements are ambiguous.
 What You'll Get to Do
-* Design and build scalable full-stack software that greatly reduces manual effort, improves quality, and creates an engaging implementation experience for customers and internal teams.
-* Use AI tools as part of your engineering stack and workflow to move faster and work smarter, with bonus value placed on experience implementing solutions that leverage generative and non-generative AI models.
-* Build across services, APIs, and modern web applications, integrating with operational, reporting, and end-user systems.
-* Collaborate closely with Product Managers, Designers, and Engineers to translate requirements into thoughtful technical solutions.
-* Generate, write, and review clean, maintainable code while contributing to code reviews and helping raise quality through testing and sound engineering practices.
-* Use AI-assisted development tools effectively and responsibly to accelerate coding, debugging, refactoring, and design exploration.
+- Design and build scalable full-stack software that greatly reduces manual effort, improves quality, and creates an engaging implementation experience for customers and internal teams.
+- Use AI tools as part of your engineering stack and workflow to move faster and work smarter, with bonus value placed on experience implementing solutions that leverage generative and non-generative AI models.
+- Build across services, APIs, and modern web applications, integrating with operational, reporting, and end-user systems.
+- Collaborate closely with Product Managers, Designers, and Engineers to translate requirements into thoughtful technical solutions.
+- Generate, write, and review clean, maintainable code while contributing to code reviews and helping raise quality through testing and sound engineering practices.
+- Use AI-assisted development tools effectively and responsibly to accelerate coding, debugging, refactoring, and design exploration.
 Skills and Experience We Value
-* Recent hands-on professional experience building and shipping production software with C# and .NET; your most recent work should be hands-on coding.
-* Full-stack development experience, with React and TypeScript strongly preferred so you can hit the ground running on our front end. Experience with other modern web technologies such as Angular or Vue is welcome and transferable.
-* Strong grounding in object-oriented design, data structures, testing, and building maintainable, reliable software.
-* Comfortable working in complex systems—including multiple services, distributed components, or other non-trivial architectures—with the ability to evaluate trade-offs and own a well-scoped feature or service end-to-end, from design through delivery.
-* AI fluency in day-to-day engineering work, including hands-on experience using AI tools in your engineering stack and workflow. Bonus value is placed on measurable outcomes from AI adoption and experience implementing solutions that leverage generative and non-generative AI models.
-* Clear communication, collaborative instincts, and a mindset of continuous learning, curiosity, and improvement that contributes to the success of the Scrum process.
-* A product mindset—you connect your work to user and business outcomes and can describe what changed because you built it, not just what you built.
-* Exposure to HCM, Workforce Management, Benefits, or Payroll domains is an asset.
+- Recent hands-on professional experience building and shipping production software with C# and .NET; your most recent work should be hands-on coding.
+- Full-stack development experience, with React and TypeScript strongly preferred so you can hit the ground running on our front end. Experience with other modern web technologies such as Angular or Vue is welcome and transferable.
+- Strong grounding in object-oriented design, data structures, testing, and building maintainable, reliable software.
+- Comfortable working in complex systems—including multiple services, distributed components, or other non-trivial architectures—with the ability to evaluate trade-offs and own a well-scoped feature or service end-to-end, from design through delivery.
+- AI fluency in day-to-day engineering work, including hands-on experience using AI tools in your engineering stack and workflow. Bonus value is placed on measurable outcomes from AI adoption and experience implementing solutions that leverage generative and non-generative AI models.
+- Clear communication, collaborative instincts, and a mindset of continuous learning, curiosity, and improvement that contributes to the success of the Scrum process.
+- A product mindset—you connect your work to user and business outcomes and can describe what changed because you built it, not just what you built.
+- Exposure to HCM, Workforce Management, Benefits, or Payroll domains is an asset.
 What Would Make You Stand Out
-* You enjoy working at the intersection of product innovation, full-stack engineering, and practical AI application.
-* You are passionate about reimagining how enterprise software implementations are delivered.
-* You thrive in collaborative environments where you can grow your technical craft while solving meaningful customer problems through AI-enabled solutions.
+- You enjoy working at the intersection of product innovation, full-stack engineering, and practical AI application.
+- You are passionate about reimagining how enterprise software implementations are delivered.
+- You thrive in collaborative environments where you can grow your technical craft while solving meaningful customer problems through AI-enabled solutions.
 What's in it for you
 Dayforce is fueled by the diversity of our talented employees. We are an equal opportunity employer and consider and embrace ALL individuals and what makes them unique. We believe our employees should be happy and healthy, with peace of mind and a sense of fulfillment.
 We encourage individuals to apply based on their passions.
@@ -1395,9 +1387,8 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-(Remote) Software Developer
-[Apply](https://harriscomputer.wd3.myworkdayjobs.com/1/job/Office---Blair/XMLNAME--Remote--Software-Developer_R0044815-6/apply?jr_id=6a5e503167b2850e77df05fc)
+          <t>(Remote) Software Developer
+Apply
 locations
 Office - Blair
 British Columbia, Canada
@@ -1437,38 +1428,38 @@
 AI &amp; Innovation Mindset
 We are committed to leveraging emerging technologies to improve how we work, serve our customers, and drive business outcomes. The successful candidate will demonstrate curiosity and a willingness to actively adopt and leverage AI tools to improve workflows, solve problems, and increase efficiency. Candidates should be comfortable using AI enabled technologies, including copilots, chat based AI assistants, and automation tools, as part of their everyday work while maintaining appropriate judgment, security, and compliance standards.
 What your impact will be:
-* Design, develop, and maintain database solutions using MSSQL.
-* Develop and maintain RESTful APIs to support various applications.
-* Write clean, scalable, and efficient code in C# using .NET Core.
-* Develop and maintain front-end applications using Angular, Typescript, HTML, and CSS.
-* Partner with cross-functional teams to define, design, and ship new features.
-* Troubleshoot and debug applications to optimize performance.
-* Take part in code reviews and contribute to the continuous improvement of the development process.
-* Stay up-to-date with the latest industry trends and technologies.
+- Design, develop, and maintain database solutions using MSSQL.
+- Develop and maintain RESTful APIs to support various applications.
+- Write clean, scalable, and efficient code in C# using .NET Core.
+- Develop and maintain front-end applications using Angular, Typescript, HTML, and CSS.
+- Partner with cross-functional teams to define, design, and ship new features.
+- Troubleshoot and debug applications to optimize performance.
+- Take part in code reviews and contribute to the continuous improvement of the development process.
+- Stay up-to-date with the latest industry trends and technologies.
 What we are looking for:
-* Associates degree in Computer Science, Engineering, or a related field.
-* Proven experience as a Software Engineer or similar role.
-* Proven proficiency in MSSQL and database design.
-* Experience with REST API development and integration.
-* Proficiency in C# and .NET Core framework.
-* Experience with Angular, Typescript, HTML, and CSS.
-* Exceptional problem-solving skills and attention to detail.
-* Excellent communication and teamwork skills.
-* Ability to work autonomously and manage multiple tasks.
+- Associates degree in Computer Science, Engineering, or a related field.
+- Proven experience as a Software Engineer or similar role.
+- Proven proficiency in MSSQL and database design.
+- Experience with REST API development and integration.
+- Proficiency in C# and .NET Core framework.
+- Experience with Angular, Typescript, HTML, and CSS.
+- Exceptional problem-solving skills and attention to detail.
+- Excellent communication and teamwork skills.
+- Ability to work autonomously and manage multiple tasks.
 What would make you stand out:
-* Experience with cloud platforms such as Azure or AWS.
-* Knowledge of Agile development methodologies.
-* Familiarity with GitHub practices and tools.
+- Experience with cloud platforms such as Azure or AWS.
+- Knowledge of Agile development methodologies.
+- Familiarity with GitHub practices and tools.
 What we can offer:
-* 3 weeks' vacation and 5 personal days
-* Comprehensive Medical, Dental, and Vision benefits starting from your first day of employment
-* Employee stock ownership and RRSP/401k matching programs
-* Lifestyle rewards
-* Remote work and more!
+- 3 weeks' vacation and 5 personal days
+- Comprehensive Medical, Dental, and Vision benefits starting from your first day of employment
+- Employee stock ownership and RRSP/401k matching programs
+- Lifestyle rewards
+- Remote work and more!
 About MACC:
 Telecommunication companies of all sizes across the United States use MACC's billing system. Our products empower clients to reach new levels of efficiency through integration and process automation. MACC's products are supported by professional and dedicated customer care teams to ensure the outstanding service our clients deserve. Plus, we offer the stability of being a growing company with more than 45 years of experience.
 About Harris:
-[Harris](https://www.harriscomputer.com/) is a leading provider of mission critical software to the public sector in North America. As a wholly owned subsidiary of Constellation Software Inc. ("CSI", symbol CSU on the TSX), Harris has become the cornerstone for CSI's investment in utility, local government, school districts, public safety, and healthcare software verticals. Our success has been realized through investments in our proprietary software and market expertise. This focus, combined with acquiring businesses that build upon or complement our offerings, has helped drive our success. Harris will continue to growth through reinvestment – both in the people and products that we offer and making investments in acquiring new businesses.
+Harris is a leading provider of mission critical software to the public sector in North America. As a wholly owned subsidiary of Constellation Software Inc. ("CSI", symbol CSU on the TSX), Harris has become the cornerstone for CSI's investment in utility, local government, school districts, public safety, and healthcare software verticals. Our success has been realized through investments in our proprietary software and market expertise. This focus, combined with acquiring businesses that build upon or complement our offerings, has helped drive our success. Harris will continue to growth through reinvestment – both in the people and products that we offer and making investments in acquiring new businesses.
 #LI-DNI</t>
         </is>
       </c>
@@ -1494,8 +1485,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-&gt; Source: pasted by user, 2026-07-20. Posted via recruiting agency hireVouch (Toronto) on behalf of an unnamed mining-tech client.
+          <t>Source: pasted by user, 2026-07-20. Posted via recruiting agency hireVouch (Toronto) on behalf of an unnamed mining-tech client.
 Forward Deployed Engineer (AI)
 Remote, Canada
 Role
@@ -1542,20 +1532,19 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t># Job Description — Data Quality Analyst (TEEMA, client: leading global retail brand)
-- **Source:** LinkedIn — https://www.linkedin.com/jobs/view/data-quality-analyst-at-teema-4442207480/
-- **Captured:** 2026-07-20 (posted ~16 minutes before capture; 3 applicants; promoted by hirer; typical review time 1 week)
-- **Location:** Vancouver, BC (Hybrid)
-- **Type:** Contract — 6-month to start
-- **Rate:** 55–58 CAD/hr
-- **Apply method:** LinkedIn Easy Apply
-- **Job poster:** Sayali Malye (TEEMA recruiter) — https://www.linkedin.com/in/sayalimalye/ — "Reducing hiring risk and time-to-hire for tech &amp; business teams across Canada &amp; USA | Permanent &amp; Contract Recruitment"
----
-## About the job
+          <t>Job Description — Data Quality Analyst (TEEMA, client: leading global retail brand)
+- Source: LinkedIn — https://www.linkedin.com/jobs/view/data-quality-analyst-at-teema-4442207480/
+- Captured: 2026-07-20 (posted ~16 minutes before capture; 3 applicants; promoted by hirer; typical review time 1 week)
+- Location: Vancouver, BC (Hybrid)
+- Type: Contract — 6-month to start
+- Rate: 55–58 CAD/hr
+- Apply method: LinkedIn Easy Apply
+- Job poster: Sayali Malye (TEEMA recruiter) — https://www.linkedin.com/in/sayalimalye/ — "Reducing hiring risk and time-to-hire for tech &amp; business teams across Canada &amp; USA | Permanent &amp; Contract Recruitment"
+About the job
 Our client, a leading global retail brand, is building out a brand-new, centralized Enterprise Data Platform. If you have a data analyst mindset, love solving data puzzles, and want to ensure data accuracy for critical business analytics and future AI use cases, this role is for you!
 This is a dedicated data validation position—not a traditional software application testing role. You will bridge the gap between complex data systems and business logic to ensure data is accurate, complete, and trusted.
 This is a 6-month contract to start - hybrid in Vancouver. Apply today to get the conversation started.
-## What You'll Do:
+What You'll Do:
 - Validate data moving between source systems and the Data Hub across raw, cleansed, and integrated layers.
 - Review requirements, business rules, source-to-target mappings, and transformation logic.
 - Design and execute QA test plans, test cases, and exception analysis.
@@ -1563,19 +1552,19 @@
 - Validate downstream reporting, dashboards, and curated datasets in Power BI.
 - Ensure sensitive information is masked, protected, and handled appropriately.
 - Help build reusable QA playbooks, reconciliation templates, and data quality standards for the future.
-## What You Bring:
+What You Bring:
 - 4+ years of Data QA / Data Validation experience (validating data between systems, reports, warehouses, or environments).
 - Strong proficiency in SQL and Excel for comparing datasets, profiling data, and investigating root causes.
 - Experience with Power BI (or similar BI tools) to validate reporting outputs.
 - Solid background in documenting test plans, test cases, defects, and test evidence.
 - Strong analytical skills to translate business requirements and transformation rules into practical validation scenarios.
 - A self-directed mindset with the ability to take ownership of your work without constant hand-holding.
-## Nice-to-Have Skills:
+Nice-to-Have Skills:
 - Experience with Databricks or Azure environments.
 - Background working with workforce, operational, or payroll data.
 - Exposure to Python or automated testing routines.
 - Experience handling sensitive or confidential compliance data.
-## What This Role Is NOT:
+What This Role Is NOT:
 - Not a traditional application/software QA role.
 - Not a senior QA Lead position.
 - Not a heavy automation or coding role at this stage.
@@ -1605,20 +1594,20 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t># Job Description (raw, verbatim)
+          <t>Job Description (raw, verbatim)
 Operations Analyst
-[CanPrev Natural Health Products Ltd.](https://ca.indeed.com/cmp/Canprev-&amp;-Orange-Naturals?campaignid=mobvjcmp&amp;from=mobviewjob&amp;tk=1ju0e2fnp2330000&amp;fromjk=6f0492fb84207a06)
+CanPrev Natural Health Products Ltd.
 North York, ON
 Hybrid work
 $55,000–$60,000 a year - Full-time
 Job details
-Here's how the job details align with your [profile](https://profile.indeed.com/).
+Here's how the job details align with your profile.
 Pay
-* $55,000–$60,000 a year
+- $55,000–$60,000 a year
 Job type
-* Full-time
+- Full-time
 Shift and schedule
-* Monday to Friday
+- Monday to Friday
 Location
 North York, ON
 Full job description
@@ -1628,56 +1617,56 @@
 The Operations Analyst supports strategic sourcing, cost management, supply continuity, and day-to-day manufacturing operations to ensure efficient, cost-effective, and reliable product supply. This role serves as a key liaison between contract manufacturers, suppliers, logistics partners, and internal stakeholders, helping maintain Just-in-Time inventory levels while driving operational excellence and margin optimization.
 Key Responsibilities:
 Sourcing, Cost Management &amp; Supply Continuity
-* Review, challenge, and negotiate proposed price increases, minimum order quantity (MOQ) changes, and commercial terms with Contract Manufacturing Organizations (CMOs).
-* Audit supplier invoices, investigate pricing discrepancies, and ensure accurate cost allocation and billing practices.
-* Maintain product cost models, margin calculators, and cost-tracking spreadsheets to identify margin risks and support profitability reviews.
-* Analyze product margins and provide recommendations on low-margin SKUs for management evaluation.
-* Identify, qualify, and onboard backup CMOs, suppliers, and alternative raw materials or components to mitigate supply chain risks.
-* Coordinate product testing, documentation, Certificates of Analysis (COAs), and approval processes for alternative materials and suppliers.
-* Source and evaluate quotations from multiple CMOs and suppliers to support new product development and product launch initiatives.
-* Support vendor performance reviews and contribute to continuous improvement initiatives across the supply network.
+- Review, challenge, and negotiate proposed price increases, minimum order quantity (MOQ) changes, and commercial terms with Contract Manufacturing Organizations (CMOs).
+- Audit supplier invoices, investigate pricing discrepancies, and ensure accurate cost allocation and billing practices.
+- Maintain product cost models, margin calculators, and cost-tracking spreadsheets to identify margin risks and support profitability reviews.
+- Analyze product margins and provide recommendations on low-margin SKUs for management evaluation.
+- Identify, qualify, and onboard backup CMOs, suppliers, and alternative raw materials or components to mitigate supply chain risks.
+- Coordinate product testing, documentation, Certificates of Analysis (COAs), and approval processes for alternative materials and suppliers.
+- Source and evaluate quotations from multiple CMOs and suppliers to support new product development and product launch initiatives.
+- Support vendor performance reviews and contribute to continuous improvement initiatives across the supply network.
 Manufacturing Operations &amp; Logistics Execution
-* Manage a portfolio of CMOs by monitoring production schedules, order timelines, and inventory requirements to maintain Just-in-Time inventory levels and prevent stockouts.
-* Conduct daily purchase order follow-ups and proactively manage production updates, delays, and issue resolution.
-* Serve as the primary operational liaison for contract manufacturers regarding quality concerns, artwork revisions, packaging updates, and invoice-related inquiries.
-* Source and negotiate competitive freight and transportation rates with third-party logistics providers (3PLs).
-* Coordinate inbound and outbound shipments of raw materials, components, labels, cartons, and finished goods.
-* Complete ERP transactions including receiving, inventory reconciliation, material consumption tracking, and production record updates.
-* Monitor open label and packaging orders, ensuring timely approvals and execution of artwork changes.
-* Route label and packaging layouts for internal review and design approval.
-* Support inventory accuracy through cycle counts, physical inventory verification, and weekly operational audits.
+- Manage a portfolio of CMOs by monitoring production schedules, order timelines, and inventory requirements to maintain Just-in-Time inventory levels and prevent stockouts.
+- Conduct daily purchase order follow-ups and proactively manage production updates, delays, and issue resolution.
+- Serve as the primary operational liaison for contract manufacturers regarding quality concerns, artwork revisions, packaging updates, and invoice-related inquiries.
+- Source and negotiate competitive freight and transportation rates with third-party logistics providers (3PLs).
+- Coordinate inbound and outbound shipments of raw materials, components, labels, cartons, and finished goods.
+- Complete ERP transactions including receiving, inventory reconciliation, material consumption tracking, and production record updates.
+- Monitor open label and packaging orders, ensuring timely approvals and execution of artwork changes.
+- Route label and packaging layouts for internal review and design approval.
+- Support inventory accuracy through cycle counts, physical inventory verification, and weekly operational audits.
 Cross-Functional Collaboration &amp; Continuous Improvement
-* Collaborate with Quality Assurance, Product Development, Finance, Regulatory, and Supply Chain teams to support product availability and operational objectives
-* Assist in identifying process improvement opportunities that enhance operational efficiency, inventory accuracy, and supplier performance
-* Develop reporting and tracking tools to improve visibility into production schedules, inventory levels, costs, and supplier performance metrics
-* Support special projects related to sourcing optimization, supply continuity, cost savings, and operational scalability
+- Collaborate with Quality Assurance, Product Development, Finance, Regulatory, and Supply Chain teams to support product availability and operational objectives
+- Assist in identifying process improvement opportunities that enhance operational efficiency, inventory accuracy, and supplier performance
+- Develop reporting and tracking tools to improve visibility into production schedules, inventory levels, costs, and supplier performance metrics
+- Support special projects related to sourcing optimization, supply continuity, cost savings, and operational scalability
 Key Qualifications
-* Bachelor's degree or diploma in Supply Chain Management, Operations Management, Business Administration, Logistics, or a related field.
-* 2+ years of experience in sourcing, supply chain, procurement, manufacturing operations, or inventory management.
-* Experience working with contract manufacturers, suppliers, and logistics providers is considered an asset.
-* Experience in consumer packaged goods (CPG), natural health products, supplements, food manufacturing, or related industries is preferred.
-* Proficiency with ERP systems, inventory management software, and Microsoft Excel.
+- Bachelor's degree or diploma in Supply Chain Management, Operations Management, Business Administration, Logistics, or a related field.
+- 2+ years of experience in sourcing, supply chain, procurement, manufacturing operations, or inventory management.
+- Experience working with contract manufacturers, suppliers, and logistics providers is considered an asset.
+- Experience in consumer packaged goods (CPG), natural health products, supplements, food manufacturing, or related industries is preferred.
+- Proficiency with ERP systems, inventory management software, and Microsoft Excel.
 Key Skills
-* Strong analytical and problem-solving skills with the ability to interpret cost and margin data.
-* Excellent negotiation and vendor management capabilities.
-* Strong organizational skills with exceptional attention to detail.
-* Ability to manage multiple priorities and deadlines in a fast-paced environment.
-* Effective communicator with strong interpersonal and relationship-building skills.
-* Proactive approach to identifying operational risks and implementing solutions.
-* Experience with inventory planning, procurement, and logistics coordination.
-* Advanced proficiency in Microsoft Excel, including data analysis and reporting.
-* Collaborative team player with the ability to work cross-functionally across multiple departments.
+- Strong analytical and problem-solving skills with the ability to interpret cost and margin data.
+- Excellent negotiation and vendor management capabilities.
+- Strong organizational skills with exceptional attention to detail.
+- Ability to manage multiple priorities and deadlines in a fast-paced environment.
+- Effective communicator with strong interpersonal and relationship-building skills.
+- Proactive approach to identifying operational risks and implementing solutions.
+- Experience with inventory planning, procurement, and logistics coordination.
+- Advanced proficiency in Microsoft Excel, including data analysis and reporting.
+- Collaborative team player with the ability to work cross-functionally across multiple departments.
 How to Apply
 Please submit your resume and a cover letter outlining your qualifications and explaining why you are the perfect fit.
 Job Type: Full-time, Permanent
 Schedule
-* Monday to Friday
-* Work Location: North York Hybrid – 4 days on site
+- Monday to Friday
+- Work Location: North York Hybrid – 4 days on site
 We thank all applicants for their interest in CanPrev Natural Health; however, only chosen applicants will be contacted. We regret that we are unable to respond to individual inquiries about application status. CanPrev Natural Health is an equal opportunity employer that fosters an inclusive, equitable, and accessible environment. Please notify us if you require accommodation at any time during the recruitment process.
 Job Type: Full-time
 Pay: $55,000.00-$60,000.00 per year
 Education:
-* Bachelor's Degree (preferred)
+- Bachelor's Degree (preferred)
 Work Location: Hybrid remote in North York, ON</t>
         </is>
       </c>
@@ -1703,17 +1692,17 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t># Job Description (raw, verbatim)
+          <t>Job Description (raw, verbatim)
 Inventory &amp; Warehouse Operations Coordinator
 MoltonRox Solutions
 7935 130 Street, Surrey, BC V3W 0H7
 $42,458.64–$55,796.75 a year - Permanent, Full-time
 Job details
 Pay
-* $42,458.64–$55,796.75 a year
+- $42,458.64–$55,796.75 a year
 Job type
-* Permanent
-* Full-time
+- Permanent
+- Full-time
 Location
 Estimated commute
 Job address
@@ -1726,67 +1715,67 @@
 This is a hands-on operational role requiring exceptional attention to detail and strong organizational skills.
 Responsibilities:
 Inventory Receiving
-* Receive incoming inventory into the ERP system
-* Verify quantities against supplier documentation
-* Investigate shortages and overages
-* Record damaged products
-* Close supplier purchase orders
-* Ensure all inventory is received within one business day
+- Receive incoming inventory into the ERP system
+- Verify quantities against supplier documentation
+- Investigate shortages and overages
+- Record damaged products
+- Close supplier purchase orders
+- Ensure all inventory is received within one business day
 Inventory Control
-* Maintain accurate inventory records
-* Perform regular cycle counts
-* Investigate inventory discrepancies
-* Maintain warehouse locations
-* Monitor inventory accuracy
+- Maintain accurate inventory records
+- Perform regular cycle counts
+- Investigate inventory discrepancies
+- Maintain warehouse locations
+- Monitor inventory accuracy
 Warehouse Coordination
-* Issue daily picking priorities
-* Coordinate warehouse workflow
-* Confirm completed shipments
-* Ensure warehouse paperwork is complete
-* Verify quantities shipped
+- Issue daily picking priorities
+- Coordinate warehouse workflow
+- Confirm completed shipments
+- Ensure warehouse paperwork is complete
+- Verify quantities shipped
 Warehouse Organization
-* Manage warehouse storage locations
-* Remove obsolete inventory
-* Monitor inventory tied to cancelled customer orders
-* Improve warehouse efficiency and organization
+- Manage warehouse storage locations
+- Remove obsolete inventory
+- Monitor inventory tied to cancelled customer orders
+- Improve warehouse efficiency and organization
 Reporting
-* Inventory accuracy reports
-* Receiving backlog
-* Open supplier purchase orders
-* Warehouse utilization
-* Inventory aging reports
+- Inventory accuracy reports
+- Receiving backlog
+- Open supplier purchase orders
+- Warehouse utilization
+- Inventory aging reports
 Required Experience
-* 3+ years in inventory control, warehouse operations or logistics
-* Experience with ERP inventory systems
-* Strong inventory reconciliation experience
-* Understanding of warehouse processes
-* Experience leading or coordinating warehouse staff
-* Strong Excel skills
+- 3+ years in inventory control, warehouse operations or logistics
+- Experience with ERP inventory systems
+- Strong inventory reconciliation experience
+- Understanding of warehouse processes
+- Experience leading or coordinating warehouse staff
+- Strong Excel skills
 Experience in wholesale distribution or supplying major retailers is preferred.
 We're Looking For Someone Who
-* Is highly organized
-* Notices small discrepancies before they become big problems
-* Enjoys creating efficient systems
-* Holds themselves accountable
-* Can prioritize work independently
-* Documents everything accurately
-* Follows standardized procedures
-* Works well with warehouse teams
-* Takes pride in maintaining inventory accuracy
+- Is highly organized
+- Notices small discrepancies before they become big problems
+- Enjoys creating efficient systems
+- Holds themselves accountable
+- Can prioritize work independently
+- Documents everything accurately
+- Follows standardized procedures
+- Works well with warehouse teams
+- Takes pride in maintaining inventory accuracy
 Success in This Role Means
-* Inventory is accurate
-* Receiving is completed on time
-* Warehouse staff know exactly what to work on
-* Shipments are picked correctly
-* The warehouse remains organized and efficient
-* Inventory can be trusted
+- Inventory is accurate
+- Receiving is completed on time
+- Warehouse staff know exactly what to work on
+- Shipments are picked correctly
+- The warehouse remains organized and efficient
+- Inventory can be trusted
 Pay: $42,458.64-$55,796.75 per year
 Application question(s):
-* When can you start work if offered a job?
-* What is your experience level in all the tasks required from this job?
-* We are located in Newton Surrey, will commute be a problem?
-* What is your typing speed?
-* What is your highest level of education? From which university and which year did you graduate?
+- When can you start work if offered a job?
+- What is your experience level in all the tasks required from this job?
+- We are located in Newton Surrey, will commute be a problem?
+- What is your typing speed?
+- What is your highest level of education? From which university and which year did you graduate?
 Work Location: In person
 Source: https://ca.indeed.com/cmp/Moltonrox-Solutions (Indeed posting)</t>
         </is>
@@ -1813,18 +1802,17 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-Customer Order &amp; Logistics Coordinator
-[MoltonRox Solutions](https://ca.indeed.com/cmp/Moltonrox-Solutions?campaignid=mobvjcmp&amp;from=mobviewjob&amp;tk=1ju0ivi6tgstq808&amp;fromjk=66079a913708672f)
+          <t>Customer Order &amp; Logistics Coordinator
+MoltonRox Solutions
 7935 130 Street, Surrey, BC V3W 0H7
 $38,637.19–$55,967.43 a year - Permanent, Full-time
 Job details
 Here's how the job details align with your profile.
 Pay
-* $38,637.19–$55,967.43 a year
+- $38,637.19–$55,967.43 a year
 Job type
-* Permanent
-* Full-time
+- Permanent
+- Full-time
 Location
 Estimated commute
 Job address
@@ -1838,65 +1826,65 @@
 If you enjoy creating order from complexity, meeting deadlines, and holding yourself to a high standard of accuracy, we'd like to hear from you.
 Responsibilities:
 Customer Order Management
-* Enter customer purchase orders accurately
-* Review PO requirements and shipping deadlines
-* Monitor all open customer orders
-* Prioritize shipments according to required delivery dates
-* Maintain accurate order records
+- Enter customer purchase orders accurately
+- Review PO requirements and shipping deadlines
+- Monitor all open customer orders
+- Prioritize shipments according to required delivery dates
+- Maintain accurate order records
 Customer Communication
-* Communicate professionally with retail buyers
-* Notify customers immediately of delays or shortages
-* Coordinate routing requests and shipping appointments
-* Respond promptly to customer inquiries
-* Build positive working relationships with customers
+- Communicate professionally with retail buyers
+- Notify customers immediately of delays or shortages
+- Coordinate routing requests and shipping appointments
+- Respond promptly to customer inquiries
+- Build positive working relationships with customers
 Shipping Coordination
-* Prepare shipping documentation
-* Book freight with carriers
-* Prepare Bills of Lading
-* Generate packing lists
-* Coordinate warehouse shipping schedules
-* Ensure all required retailer documentation is completed
+- Prepare shipping documentation
+- Book freight with carriers
+- Prepare Bills of Lading
+- Generate packing lists
+- Coordinate warehouse shipping schedules
+- Ensure all required retailer documentation is completed
 After Shipment
-* Confirm shipments have left on schedule
-* Send invoices promptly after shipment
-* Maintain complete shipment records
-* Provide proof of shipment and tracking when required
+- Confirm shipments have left on schedule
+- Send invoices promptly after shipment
+- Maintain complete shipment records
+- Provide proof of shipment and tracking when required
 Reporting
-* Daily shipping schedule
-* Open order report
-* Late shipment report
-* Customer communication log
+- Daily shipping schedule
+- Open order report
+- Late shipment report
+- Customer communication log
 Required Experience
-* 3+ years in logistics, customer service, order management, or supply chain
-* Experience working with purchase orders
-* Experience coordinating freight shipments
-* Experience using ERP or inventory software
-* Strong Microsoft Excel skills
-* Excellent written and verbal communication
+- 3+ years in logistics, customer service, order management, or supply chain
+- Experience working with purchase orders
+- Experience coordinating freight shipments
+- Experience using ERP or inventory software
+- Strong Microsoft Excel skills
+- Excellent written and verbal communication
 Experience supplying large retailers such as Walmart, Costco, Target, Kroger, Home Depot, Lowe's or similar is considered a significant asset.
 We're Looking For Someone Who
-* Never lets deadlines slip
-* Communicates problems early
-* Is exceptionally organized
-* Keeps accurate records
-* Follows procedures consistently
-* Can manage multiple priorities
-* Takes ownership of mistakes and resolves them
-* Doesn't rely on memory to manage work
-* Enjoys checklists and process improvement
+- Never lets deadlines slip
+- Communicates problems early
+- Is exceptionally organized
+- Keeps accurate records
+- Follows procedures consistently
+- Can manage multiple priorities
+- Takes ownership of mistakes and resolves them
+- Doesn't rely on memory to manage work
+- Enjoys checklists and process improvement
 Success in This Role Means
-* Orders ship on time
-* Customers are informed before problems occur
-* Invoices are sent immediately after shipment
-* Documentation is complete and accurate
-* Buyers have confidence in working with our company
+- Orders ship on time
+- Customers are informed before problems occur
+- Invoices are sent immediately after shipment
+- Documentation is complete and accurate
+- Buyers have confidence in working with our company
 Pay: $38,637.19-$55,967.43 per year
 Application question(s):
-* When can you start work if offered a job?
-* What is your experience level in all the tasks required from this job?
-* We are located in Newton Surrey, will commute be a problem?
-* What is your typing speed?
-* What is your highest level of education? From which university and which year did you graduate?
+- When can you start work if offered a job?
+- What is your experience level in all the tasks required from this job?
+- We are located in Newton Surrey, will commute be a problem?
+- What is your typing speed?
+- What is your highest level of education? From which university and which year did you graduate?
 Work Location: In person</t>
         </is>
       </c>
@@ -1922,8 +1910,8 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t># Job Description — Waabi, Applied Scientist (verbatim)
-&gt; Captured 2026-07-21. Posting: Toronto, ON / San Francisco, CA / Pittsburgh, PA / Remote US &amp; Canada. Software – Autonomy &amp; Algorithms / Full-time / Hybrid.
+          <t>Job Description — Waabi, Applied Scientist (verbatim)
+Captured 2026-07-21. Posting: Toronto, ON / San Francisco, CA / Pittsburgh, PA / Remote US &amp; Canada. Software – Autonomy &amp; Algorithms / Full-time / Hybrid.
 Applied Scientist
 Toronto, ON / San Francisco, CA / Pittsburgh, PA / Remote US &amp; Canada
 Software – Autonomy &amp; Algorithms / Full-time / Hybrid
@@ -1985,8 +1973,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-Data Scientist
+          <t>Data Scientist
 Location:
 Burnaby, BC, CA, V5H 3Z7 Mississauga, ON, CA Calgary, AB, CA Toronto, ON, CA Edmonton, AB, CA Vancouver, BC, CA
 Req ID:  53658
@@ -2001,35 +1988,35 @@
 What you'll do
 As a Data Scientist, you'll work closely with stakeholders and software engineers to identify and implement scalable data architectures, transform raw data into actionable insights, and create compelling visualizations that drive business decisions across TELUS.
 Your Responsibilities:
-* Data Architecture &amp; Engineering: Design and build robust data pipelines and architectures on Google Cloud Platform (GCP), leveraging BigQuery, Workflows, Cloud Scheduler, Dataproc, and Batch jobs. Establish scalable ETL/ELT processes that efficiently ingest, transform, and prepare data from diverse sources for analytics and reporting. Build and manage GCP resources using Pulumi and YAML configurations, and maintain code in GitHub.
-* Advanced Analytics &amp; Insights: Conduct in-depth exploratory data analysis and apply statistical methods, machine learning techniques, and AI-driven analytics to uncover patterns, trends, and actionable business insights. Develop analytical models and leverage AI capabilities to support strategic decision-making and operational improvements across key business metrics.
-* Data Visualization &amp; Dashboards: Design and build intuitive, visually compelling dashboards and reports in Looker Studio that communicate complex data stories to diverse stakeholders. Create data visualizations with a strong eye for clarity, aesthetics, and user experience that enable self-service analytics.
-* GCP Platform Expertise: Leverage GCP's data ecosystem (BigQuery, Workflows, Cloud Scheduler, Dataproc, Batch, and Vertex AI) to optimize query performance, reduce costs, and enable real-time analytics. Implement best practices for data governance, security, and scalability within GCP environments.
-* Collaboration and Mentoring: Work with business teams and stakeholders to understand data requirements and translate business questions into analytical solutions. Document analytical findings and architectural decisions clearly, and mentor team members on data best practices.
+- Data Architecture &amp; Engineering: Design and build robust data pipelines and architectures on Google Cloud Platform (GCP), leveraging BigQuery, Workflows, Cloud Scheduler, Dataproc, and Batch jobs. Establish scalable ETL/ELT processes that efficiently ingest, transform, and prepare data from diverse sources for analytics and reporting. Build and manage GCP resources using Pulumi and YAML configurations, and maintain code in GitHub.
+- Advanced Analytics &amp; Insights: Conduct in-depth exploratory data analysis and apply statistical methods, machine learning techniques, and AI-driven analytics to uncover patterns, trends, and actionable business insights. Develop analytical models and leverage AI capabilities to support strategic decision-making and operational improvements across key business metrics.
+- Data Visualization &amp; Dashboards: Design and build intuitive, visually compelling dashboards and reports in Looker Studio that communicate complex data stories to diverse stakeholders. Create data visualizations with a strong eye for clarity, aesthetics, and user experience that enable self-service analytics.
+- GCP Platform Expertise: Leverage GCP's data ecosystem (BigQuery, Workflows, Cloud Scheduler, Dataproc, Batch, and Vertex AI) to optimize query performance, reduce costs, and enable real-time analytics. Implement best practices for data governance, security, and scalability within GCP environments.
+- Collaboration and Mentoring: Work with business teams and stakeholders to understand data requirements and translate business questions into analytical solutions. Document analytical findings and architectural decisions clearly, and mentor team members on data best practices.
 Qualifications
 What you bring
-* Master's degree in Computer Science, Data Science, Statistics, Engineering, or a related quantitative discipline — or a PhD in a relevant field.
-* 3+ years of experience designing and implementing data architectures and analytics solutions in production environments, delivering measurable business impact.
-* Advanced proficiency in Google Cloud Platform (GCP), with hands-on experience in BigQuery, Workflows, Cloud Scheduler, Dataproc, and Batch jobs.
-* Expert-level experience with Looker Studio for creating dashboards, reports, and data visualizations that drive business insights and support decision-making.
-* Strong foundation in data architecture and ETL/ELT design, with the ability to optimize data pipelines for performance, scalability, and cost efficiency.
-* Demonstrated expertise in data visualization and analytics, with a keen eye for designing clear, compelling, and actionable insights that resonate with both technical and business audiences.
-* Experience working in GitHub, building and managing GCP resources using Pulumi and YAML configurations.
-* Strong SQL skills and experience working with large-scale datasets; proficiency in data modeling and dimensional design.
-* Proven experience analyzing structured and unstructured data using statistical methods, exploratory data analysis, and machine learning techniques to drive insights.
-* Proficiency in Python or similar languages for data processing and analytics.
-* Experience leveraging AI capabilities and tools (such as Vertex AI) to build machine learning models and AI solutions that enhance analytical capabilities.
-* Experience deploying and monitoring data solutions in production, with familiarity in CI/CD, version control, and cloud infrastructure best practices.
-* Strong ability to translate business questions into analytical frameworks and communicate findings effectively with both technical and non-technical stakeholders.
+- Master's degree in Computer Science, Data Science, Statistics, Engineering, or a related quantitative discipline — or a PhD in a relevant field.
+- 3+ years of experience designing and implementing data architectures and analytics solutions in production environments, delivering measurable business impact.
+- Advanced proficiency in Google Cloud Platform (GCP), with hands-on experience in BigQuery, Workflows, Cloud Scheduler, Dataproc, and Batch jobs.
+- Expert-level experience with Looker Studio for creating dashboards, reports, and data visualizations that drive business insights and support decision-making.
+- Strong foundation in data architecture and ETL/ELT design, with the ability to optimize data pipelines for performance, scalability, and cost efficiency.
+- Demonstrated expertise in data visualization and analytics, with a keen eye for designing clear, compelling, and actionable insights that resonate with both technical and business audiences.
+- Experience working in GitHub, building and managing GCP resources using Pulumi and YAML configurations.
+- Strong SQL skills and experience working with large-scale datasets; proficiency in data modeling and dimensional design.
+- Proven experience analyzing structured and unstructured data using statistical methods, exploratory data analysis, and machine learning techniques to drive insights.
+- Proficiency in Python or similar languages for data processing and analytics.
+- Experience leveraging AI capabilities and tools (such as Vertex AI) to build machine learning models and AI solutions that enhance analytical capabilities.
+- Experience deploying and monitoring data solutions in production, with familiarity in CI/CD, version control, and cloud infrastructure best practices.
+- Strong ability to translate business questions into analytical frameworks and communicate findings effectively with both technical and non-technical stakeholders.
 Salary Range:  $86,000-$160,000
 Performance Bonus or Sales Incentive Plan:  15%
 Actual total compensation will be determined based on factors such as knowledge, skills, performance and experience. We encourage all qualified candidates to apply, even if the posted salary range doesn't match your expectations. We're open to discussing competitive compensation packages tailored to your experience level and expertise. TELUS offers rewarding benefits, which may vary per job function, such as:
-* Comprehensive total rewards package highlighting competitive salary and bonus structures, minimum 3 weeks of vacation, and flexible benefits plan to meet the needs of you and your family
-* Flexibility to work in-office, virtually or a combination of both
-* Generous company matched pension and share purchase programs
-* Opportunity to give back to communities in which we work, live and serve
-* Career growth and learning &amp; development opportunities to develop your skills
-* And much more …
+- Comprehensive total rewards package highlighting competitive salary and bonus structures, minimum 3 weeks of vacation, and flexible benefits plan to meet the needs of you and your family
+- Flexibility to work in-office, virtually or a combination of both
+- Generous company matched pension and share purchase programs
+- Opportunity to give back to communities in which we work, live and serve
+- Career growth and learning &amp; development opportunities to develop your skills
+- And much more …
 Job Type:  This is for a current vacancy</t>
         </is>
       </c>
@@ -2055,10 +2042,9 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t># Job Description (verbatim)
-Data Analyst
+          <t>Data Analyst
 Full Time, Permanent
-[Apply](https://join.specsavers.com/ca/Workflow?workflowId=5e34479a-b5e7-4ac9-8595-2bf0fdcc96a3&amp;vacancyId=13749)Shortlist
+ApplyShortlist
 Share
 The role
 Location: This hybrid role requires 2-3 days on-site at our Burnaby, BC office.
@@ -2070,49 +2056,49 @@
 The Data Analyst delivers Power BI visualizations and dashboards that tell a story using data, drive action, and deliver value to the business. You work within a cross-functional product team, with support from product owners, business analysts, data engineers and data scientists where needed. You will also support the business in the transformation by contributing towards beginners' sessions, drop-ins, and show-and-tell sessions demonstrating the capability of Power BI and wider visualization best practice.
 Key Responsibilities
 Deliver:
-* Work with stakeholders and other data team colleagues to understand the data and insights needed to address business questions and challenges
-* Use visualization techniques to tell data stories, delivering insight to the business in a compelling way
-* Design and implement analytics reporting dashboards and visualizations using SQL and Power BI
-* Work with engineers to model, reshape and prepare data to optimize dashboard performance
-* Collaborate within the wider Data Team and Technology where required for the successful end-to-end delivery of the analytics solution
-* Work with business end-users to ensure the best user experience
-* Manage stakeholder expectations on analytical work by providing regular written and verbal communications, building trust, and forming close working relationships
+- Work with stakeholders and other data team colleagues to understand the data and insights needed to address business questions and challenges
+- Use visualization techniques to tell data stories, delivering insight to the business in a compelling way
+- Design and implement analytics reporting dashboards and visualizations using SQL and Power BI
+- Work with engineers to model, reshape and prepare data to optimize dashboard performance
+- Collaborate within the wider Data Team and Technology where required for the successful end-to-end delivery of the analytics solution
+- Work with business end-users to ensure the best user experience
+- Manage stakeholder expectations on analytical work by providing regular written and verbal communications, building trust, and forming close working relationships
 Transform:
-* Be a subject matter expert in visualization and Power BI
-* Continually improve your own knowledge, including participating in the Specsavers data visualization and storytelling training programme, and other training events
-* Share your knowledge with less experienced colleagues
-* Keep up to date on the latest analytics &amp; visualization innovation, share ideas and highlight opportunities to adopt them
-* Encourage use of data visualization and storytelling in decision making
+- Be a subject matter expert in visualization and Power BI
+- Continually improve your own knowledge, including participating in the Specsavers data visualization and storytelling training programme, and other training events
+- Share your knowledge with less experienced colleagues
+- Keep up to date on the latest analytics &amp; visualization innovation, share ideas and highlight opportunities to adopt them
+- Encourage use of data visualization and storytelling in decision making
 What We're Looking For
-* 3-5 years of experience as a Data Analyst across the data lifecycle, from data modelling and transformation to visualization and analytics, leveraging SQL, Power BI, Databricks, and related tools.
-* Experience manipulating. transforming and cleansing data, and building compelling visualizations, ideally in Power BI
-* Experience delivering reports, dashboards, or visualization projects in a business context
-* Intermediate SQL for analytics
-* Able to convey complex concepts to non-technical audiences in a succinct and accessible way
-* A collaborative approach to working, with good relationship building skills
-* Capability in DAX, Power Query or equivalent
+- 3-5 years of experience as a Data Analyst across the data lifecycle, from data modelling and transformation to visualization and analytics, leveraging SQL, Power BI, Databricks, and related tools.
+- Experience manipulating. transforming and cleansing data, and building compelling visualizations, ideally in Power BI
+- Experience delivering reports, dashboards, or visualization projects in a business context
+- Intermediate SQL for analytics
+- Able to convey complex concepts to non-technical audiences in a succinct and accessible way
+- A collaborative approach to working, with good relationship building skills
+- Capability in DAX, Power Query or equivalent
 Nice-to-have:
-* Experience working with stakeholders to refine requirements and design outputs
-* Mentoring or coaching experience
-* Experience in Python or PySpark
-* Experience working in any capacity in retail or ecommerce, marketing, supply chain, healthcare or other regulated environments such as telco, financial services and utilities.
+- Experience working with stakeholders to refine requirements and design outputs
+- Mentoring or coaching experience
+- Experience in Python or PySpark
+- Experience working in any capacity in retail or ecommerce, marketing, supply chain, healthcare or other regulated environments such as telco, financial services and utilities.
 Compensation: $80,000 - $95,000 base salary, plus quarterly bonus, profit sharing, and benefits. Actual compensation will be determined based on experience
 Speccies' Benefits
-* 4 weeks of vacation and 1 paid volunteer day per year
-* 1 extra paid day off plus an eyecare voucher to celebrate your birthday.
-* Health and dental benefits, RRSP matching and a Healthcare Spending Account active from your first day.
-* Mental health and wellbeing support, including $3,000 annually for practitioner care and access to our Employee Assistance Program.
-* Quarterly bonuses, based on your performance.
-* Annual Profit Share program to recognize your part in Specsavers' success.
-* Free parking, access to the building gym, and a fully stocked kitchen with snacks and coffee/tea.
-* On‑site wellness offerings in-office, including RMT and yoga sessions.
-* Team and company social events, including holiday and annual celebrations.
+- 4 weeks of vacation and 1 paid volunteer day per year
+- 1 extra paid day off plus an eyecare voucher to celebrate your birthday.
+- Health and dental benefits, RRSP matching and a Healthcare Spending Account active from your first day.
+- Mental health and wellbeing support, including $3,000 annually for practitioner care and access to our Employee Assistance Program.
+- Quarterly bonuses, based on your performance.
+- Annual Profit Share program to recognize your part in Specsavers' success.
+- Free parking, access to the building gym, and a fully stocked kitchen with snacks and coffee/tea.
+- On‑site wellness offerings in-office, including RMT and yoga sessions.
+- Team and company social events, including holiday and annual celebrations.
 Behaviours We Value
-* Collaborative: We work together as one Specsavers to deliver on our purpose
-* Curious: We question, explore and seek out diverse perspectives to develop our knowledge and understanding
-* Courageous: We challenge the status quo, we experiment with good ideas, and we are brave, bold and fast in our decision making
-* Compassionate: We care, support and help each other
-* Commercial: We treat money wisely and make decisions that are good for our customers, our partners, our people and for the long term
+- Collaborative: We work together as one Specsavers to deliver on our purpose
+- Curious: We question, explore and seek out diverse perspectives to develop our knowledge and understanding
+- Courageous: We challenge the status quo, we experiment with good ideas, and we are brave, bold and fast in our decision making
+- Compassionate: We care, support and help each other
+- Commercial: We treat money wisely and make decisions that are good for our customers, our partners, our people and for the long term
 We hope that in applying with us, you value these things as well!
 Our Hybrid Work Model
 Experience the best of both worlds. At Specsavers, we embrace a hybrid approach that balances in-office collaboration with the flexibility to work from home. We come together in office two to three days a week to connect, innovate, and keep our culture thriving.

</xml_diff>

<commit_message>
tracker: add Salary column to application-tracker.xlsx
Column E between Status and Job Description; backfilled all 21 rows
with posted ranges from the JDs, or researched estimates (Glassdoor/
levels.fyi) where the posting names none. Script add command now
takes --salary.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/application-tracker.xlsx
+++ b/application-tracker.xlsx
@@ -69,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -77,6 +77,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -447,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -487,7 +490,14 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>The Job Description column holds the posting verbatim; the full application artifacts live on git branch &lt;slug&gt; under applications/&lt;slug&gt;/.</t>
+          <t>Salary is the posted range from the JD when the posting names one, otherwise a researched estimate marked (est., &lt;source&gt;).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>The Job Description column holds the posting as plain text; the original markdown and all application artifacts live on git branch &lt;slug&gt; under applications/&lt;slug&gt;/.</t>
         </is>
       </c>
     </row>
@@ -502,14 +512,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="90" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="90" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -535,6 +546,11 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
           <t>Job Description</t>
         </is>
       </c>
@@ -558,7 +574,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>$135K-155K CAD (posted)</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Machine Learning Engineer, Operations Technology
 Location: Toronto, Ontario, Canada
@@ -620,7 +641,12 @@
           <t>Interview</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Not posted ("competitive")</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>AI Engineer (Speech and Audio Systems) — FGF Brands
 Primary Job Location: CA-ON-Greater Toronto Area
@@ -677,7 +703,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>CA$95K-125K (est., Glassdoor)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>AI Engineer
 About Armilla AI
@@ -739,7 +770,12 @@
           <t>Rejected</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>CA$90K-120K total (est., levels.fyi/Glassdoor)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>JOB ID -SAPXJP00084142
 Request Title
@@ -794,7 +830,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>$77.3K-111.1K CAD (posted)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Software Developer
 Apply
@@ -901,7 +942,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>$54K-62K annualized (posted)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Full Stack Developer Intern (Fall 2026) — GeoComply
 Vancouver, BC
@@ -1002,7 +1048,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>$85K-100K + 10% bonus (posted)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Business Intelligence &amp; Analytics Specialist
 Job Category: Information Technology
@@ -1056,7 +1107,12 @@
           <t>Rejected</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>$40/hr incorporated (offered)</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>AI/ML Platform Developer (Contract) — via Apex Systems
 Client: SAP
@@ -1114,7 +1170,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>CAD 90K-115K (est., Glassdoor)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Data Scientist, Analytics (Remote, Canada)
 Remote (Canada)
@@ -1175,7 +1236,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>$114.8K-191.8K CAD base (posted)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Software Development Engineer, Middle Mile P&amp;O
 Job ID: 3185274 | Amazon Development Centre Canada ULC
@@ -1233,7 +1299,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>$77.7K-107.9K CAD (posted)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Data Analyst EA SPORTS™ FC (Game Development Analytics)
 - Home
@@ -1312,7 +1383,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>$92.6K-142.6K CAD (posted)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Job Description (raw, verbatim)
 Software Developer III
@@ -1385,7 +1461,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>$40K-65K (posted)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>(Remote) Software Developer
 Apply
@@ -1483,7 +1564,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>CAD 100K-130K (est., Glassdoor)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Source: pasted by user, 2026-07-20. Posted via recruiting agency hireVouch (Toronto) on behalf of an unnamed mining-tech client.
 Forward Deployed Engineer (AI)
@@ -1530,7 +1616,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>$55-58 CAD/hr (posted)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Job Description — Data Quality Analyst (TEEMA, client: leading global retail brand)
 - Source: LinkedIn — https://www.linkedin.com/jobs/view/data-quality-analyst-at-teema-4442207480/
@@ -1592,7 +1683,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>$55K-60K (posted)</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>Job Description (raw, verbatim)
 Operations Analyst
@@ -1690,7 +1786,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>$42.5K-55.8K (posted)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>Job Description (raw, verbatim)
 Inventory &amp; Warehouse Operations Coordinator
@@ -1800,7 +1901,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>$38.6K-56K (posted)</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>Customer Order &amp; Logistics Coordinator
 MoltonRox Solutions
@@ -1908,7 +2014,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>US $128K-184K + equity/bonus (posted)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>Job Description — Waabi, Applied Scientist (verbatim)
 Captured 2026-07-21. Posting: Toronto, ON / San Francisco, CA / Pittsburgh, PA / Remote US &amp; Canada. Software – Autonomy &amp; Algorithms / Full-time / Hybrid.
@@ -1971,7 +2082,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>$86K-160K + 15% bonus (posted)</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>Data Scientist
 Location:
@@ -2040,7 +2156,12 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>$80K-95K + bonus + profit share (posted)</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Data Analyst
 Full Time, Permanent

</xml_diff>

<commit_message>
tracker: salary column as plain ranges only (e.g. 80K to 95K)
No source tags, bonus notes, or currency symbols per user preference;
hourly roles as X to Y per hour, USD suffix only for non-CAD.
Script --salary help and README tab updated to the same convention.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/application-tracker.xlsx
+++ b/application-tracker.xlsx
@@ -69,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -77,6 +77,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -559,27 +562,27 @@
       <c r="A2" s="4" t="n">
         <v>46210</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>HelloFresh</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Machine Learning Engineer</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>$135K-155K CAD (posted)</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>135K to 155K</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Machine Learning Engineer, Operations Technology
 Location: Toronto, Ontario, Canada
@@ -626,27 +629,27 @@
       <c r="A3" s="4" t="n">
         <v>46210</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>FGF Brands</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>AI Engineer (Speech &amp; Audio Systems)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Interview</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>Not posted ("competitive")</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Not posted</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>AI Engineer (Speech and Audio Systems) — FGF Brands
 Primary Job Location: CA-ON-Greater Toronto Area
@@ -688,27 +691,27 @@
       <c r="A4" s="4" t="n">
         <v>46216</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Armilla AI</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>AI Engineer</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>CA$95K-125K (est., Glassdoor)</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>95K to 125K</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>AI Engineer
 About Armilla AI
@@ -755,27 +758,27 @@
       <c r="A5" s="4" t="n">
         <v>46216</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Developer T2 (Platform Eng &amp; AI/ML)</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>CA$90K-120K total (est., levels.fyi/Glassdoor)</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>90K to 120K</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>JOB ID -SAPXJP00084142
 Request Title
@@ -815,27 +818,27 @@
       <c r="A6" s="4" t="n">
         <v>46216</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>UBC (Faculty of Medicine)</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Software Developer (JR25262)</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>$77.3K-111.1K CAD (posted)</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>77.3K to 111.1K</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Software Developer
 Apply
@@ -927,27 +930,27 @@
       <c r="A7" s="4" t="n">
         <v>46217</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>GeoComply</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Full Stack Developer Intern (Fall 2026)</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>$54K-62K annualized (posted)</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>54K to 62K</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Full Stack Developer Intern (Fall 2026) — GeoComply
 Vancouver, BC
@@ -1033,27 +1036,27 @@
       <c r="A8" s="4" t="n">
         <v>46217</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Nature's Path Foods</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Business Intelligence &amp; Analytics Specialist</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>$85K-100K + 10% bonus (posted)</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>85K to 100K</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Business Intelligence &amp; Analytics Specialist
 Job Category: Information Technology
@@ -1092,27 +1095,27 @@
       <c r="A9" s="4" t="n">
         <v>46217</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Apex Systems (client: SAP)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>AI/ML Platform Developer (BDC Foundation Infra)</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>$40/hr incorporated (offered)</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>40 per hour</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>AI/ML Platform Developer (Contract) — via Apex Systems
 Client: SAP
@@ -1155,27 +1158,27 @@
       <c r="A10" s="4" t="n">
         <v>46223</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>ZestyAI</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Data Scientist, Analytics</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>CAD 90K-115K (est., Glassdoor)</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>90K to 115K</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Data Scientist, Analytics (Remote, Canada)
 Remote (Canada)
@@ -1221,27 +1224,27 @@
       <c r="A11" s="4" t="n">
         <v>46223</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>SDE II, Middle Mile P&amp;O (REO)</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>$114.8K-191.8K CAD base (posted)</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>114.8K to 191.8K</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Software Development Engineer, Middle Mile P&amp;O
 Job ID: 3185274 | Amazon Development Centre Canada ULC
@@ -1284,27 +1287,27 @@
       <c r="A12" s="4" t="n">
         <v>46223</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Electronic Arts</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Data Analyst, EA SPORTS FC (Game Development Analytics)</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>$77.7K-107.9K CAD (posted)</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>77.7K to 107.9K</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Data Analyst EA SPORTS™ FC (Game Development Analytics)
 - Home
@@ -1368,27 +1371,27 @@
       <c r="A13" s="4" t="n">
         <v>46223</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Dayforce</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Software Developer III</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>$92.6K-142.6K CAD (posted)</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>92.6K to 142.6K</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Job Description (raw, verbatim)
 Software Developer III
@@ -1446,27 +1449,27 @@
       <c r="A14" s="4" t="n">
         <v>46223</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>MACC (Harris / Constellation)</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Software Developer (Remote)</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>$40K-65K (posted)</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>40K to 65K</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>(Remote) Software Developer
 Apply
@@ -1549,27 +1552,27 @@
       <c r="A15" s="4" t="n">
         <v>46223</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>hireVouch (client: mining-tech co)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Forward Deployed Engineer (AI)</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>CAD 100K-130K (est., Glassdoor)</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>100K to 130K</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Source: pasted by user, 2026-07-20. Posted via recruiting agency hireVouch (Toronto) on behalf of an unnamed mining-tech client.
 Forward Deployed Engineer (AI)
@@ -1601,27 +1604,27 @@
       <c r="A16" s="4" t="n">
         <v>46223</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>TEEMA (client: global retail brand)</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Data Quality Analyst</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>$55-58 CAD/hr (posted)</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>55 to 58 per hour</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Job Description — Data Quality Analyst (TEEMA, client: leading global retail brand)
 - Source: LinkedIn — https://www.linkedin.com/jobs/view/data-quality-analyst-at-teema-4442207480/
@@ -1668,27 +1671,27 @@
       <c r="A17" s="4" t="n">
         <v>46223</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>CanPrev Natural Health Products</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Operations Analyst</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>$55K-60K (posted)</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>55K to 60K</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Job Description (raw, verbatim)
 Operations Analyst
@@ -1771,27 +1774,27 @@
       <c r="A18" s="4" t="n">
         <v>46223</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>MoltonRox Solutions</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Inventory &amp; Warehouse Operations Coordinator</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>$42.5K-55.8K (posted)</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>42.5K to 55.8K</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Job Description (raw, verbatim)
 Inventory &amp; Warehouse Operations Coordinator
@@ -1886,27 +1889,27 @@
       <c r="A19" s="4" t="n">
         <v>46223</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>MoltonRox Solutions</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Customer Order &amp; Logistics Coordinator</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>$38.6K-56K (posted)</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>38.6K to 56K</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>Customer Order &amp; Logistics Coordinator
 MoltonRox Solutions
@@ -1999,27 +2002,27 @@
       <c r="A20" s="4" t="n">
         <v>46224</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Waabi</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Applied Scientist (Evaluation)</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>US $128K-184K + equity/bonus (posted)</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>128K to 184K USD</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Job Description — Waabi, Applied Scientist (verbatim)
 Captured 2026-07-21. Posting: Toronto, ON / San Francisco, CA / Pittsburgh, PA / Remote US &amp; Canada. Software – Autonomy &amp; Algorithms / Full-time / Hybrid.
@@ -2067,27 +2070,27 @@
       <c r="A21" s="4" t="n">
         <v>46224</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>TELUS</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Data Scientist (Systems Simplification Innovation Hub)</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>$86K-160K + 15% bonus (posted)</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>86K to 160K</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>Data Scientist
 Location:
@@ -2141,27 +2144,27 @@
       <c r="A22" s="4" t="n">
         <v>46225</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Specsavers Canada</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Data Analyst</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>$80K-95K + bonus + profit share (posted)</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>80K to 95K</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Data Analyst
 Full Time, Permanent

</xml_diff>